<commit_message>
rsa without matching partners
</commit_message>
<xml_diff>
--- a/RSA analysis/All excluded subs after rsa.xlsx
+++ b/RSA analysis/All excluded subs after rsa.xlsx
@@ -542,7 +542,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -554,7 +554,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -566,7 +566,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -578,7 +578,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>65</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -590,7 +590,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -602,7 +602,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -614,7 +614,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -626,7 +626,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -638,7 +638,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -650,7 +650,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -662,7 +662,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -674,7 +674,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -686,7 +686,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -844,7 +844,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -868,7 +868,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>78</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>65</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -892,7 +892,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -904,7 +904,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>68</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>75</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -952,7 +952,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -964,7 +964,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1170,7 +1170,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1194,7 +1194,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1206,7 +1206,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1242,7 +1242,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1266,7 +1266,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1278,7 +1278,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>57</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1290,7 +1290,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>49</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1496,7 +1496,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>78</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1532,7 +1532,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1544,7 +1544,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1568,7 +1568,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>75</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1580,7 +1580,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1604,7 +1604,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1616,7 +1616,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1640,7 +1640,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>